<commit_message>
Cost estimate v2: fill VM and disk rates
Rates from the Microsoft Azure Retail Prices API, East US pay-as-you-go,
30 Sep 2026: Standard_D2s_v5 Windows $0.188/hr ($137.24/month at 730 h),
Premium SSD P10 LRS $19.71/month. Total per seat for 6 hours: $1.81
(Azure $1.34 + Microsoft 365 E5 licence $0.48).
</commit_message>
<xml_diff>
--- a/cost-estimate/KnowYourData_Cost_Estimation-v2.xlsx
+++ b/cost-estimate/KnowYourData_Cost_Estimation-v2.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AI-Testing-Workspace\Cosmos-Labs\UC2-Know-Your-Data-Purview\06-Retest\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AI-Testing-Workspace\Cosmos-Labs\UC2-Know-Your-Data-Purview\06-Retest\uc2-repo\cost-estimate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAB9A745-115C-4BFC-AF4C-AB0C6AF3EA72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F46E7106-2F79-4621-8F98-C1C7E1C81099}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="1" xr2:uid="{B6782F7B-B403-4565-A0E7-E988FF44DA43}"/>
   </bookViews>
@@ -229,16 +229,16 @@
     <t>Standard D2s v5 (2 vcpus, 8 GiB memory)</t>
   </si>
   <si>
-    <t>Premium SSD LRS, ~128 GB</t>
-  </si>
-  <si>
     <t>Microsoft 365 E5 licence (per user)</t>
   </si>
   <si>
     <t>1 licence, held for the lab period</t>
   </si>
   <si>
-    <t>VM confirmed Standard_D2s_v5 and disk Premium_LRS from this repo's own DeploymentPackage/deploy-01.json, 30 Sep 2026. VM and disk Cost/Month are blank - confirm current East US pay-as-you-go rates and enter them.</t>
+    <t>Premium SSD P10 LRS, 128 GiB</t>
+  </si>
+  <si>
+    <t>Rates: Microsoft Azure Retail Prices API, East US pay-as-you-go, 30 Sep 2026 - D2s v5 Windows $0.188/hr (x730 = $137.24/month), Premium SSD P10 LRS $19.71/month. VM and disk confirmed from this repo's DeploymentPackage/deploy-01.json.</t>
   </si>
 </sst>
 </file>
@@ -1246,6 +1246,42 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -1312,46 +1348,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1362,12 +1358,16 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1827,7 +1827,7 @@
       </c>
       <c r="C7" s="56">
         <f>'Cost-Estimation'!H18</f>
-        <v>0.50541666666666663</v>
+        <v>1.8133333333333335</v>
       </c>
       <c r="D7" s="36">
         <v>6</v>
@@ -1856,7 +1856,7 @@
       </c>
       <c r="C8" s="57">
         <f>'Cost-Estimation'!H18</f>
-        <v>0.50541666666666663</v>
+        <v>1.8133333333333335</v>
       </c>
       <c r="D8" s="39">
         <f>SUM(D7)</f>
@@ -1891,7 +1891,7 @@
       </c>
       <c r="C10" s="58">
         <f>C8/F7</f>
-        <v>0.50541666666666663</v>
+        <v>1.8133333333333335</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
@@ -1928,80 +1928,80 @@
       <c r="J12" s="2"/>
     </row>
     <row r="13" spans="1:10" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="107"/>
-      <c r="B13" s="108" t="s">
+      <c r="A13" s="105"/>
+      <c r="B13" s="106" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="106"/>
-      <c r="D13" s="106"/>
-      <c r="E13" s="106"/>
-      <c r="F13" s="105"/>
-      <c r="G13" s="105"/>
-      <c r="H13" s="105"/>
-      <c r="I13" s="105"/>
-      <c r="J13" s="105"/>
+      <c r="C13" s="104"/>
+      <c r="D13" s="104"/>
+      <c r="E13" s="104"/>
+      <c r="F13" s="111"/>
+      <c r="G13" s="111"/>
+      <c r="H13" s="111"/>
+      <c r="I13" s="111"/>
+      <c r="J13" s="111"/>
     </row>
     <row r="14" spans="1:10" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="107"/>
-      <c r="B14" s="109" t="s">
+      <c r="A14" s="105"/>
+      <c r="B14" s="107" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="104"/>
-      <c r="D14" s="104"/>
-      <c r="E14" s="104"/>
-      <c r="F14" s="105"/>
-      <c r="G14" s="105"/>
-      <c r="H14" s="105"/>
-      <c r="I14" s="105"/>
-      <c r="J14" s="105"/>
+      <c r="C14" s="108"/>
+      <c r="D14" s="108"/>
+      <c r="E14" s="108"/>
+      <c r="F14" s="111"/>
+      <c r="G14" s="111"/>
+      <c r="H14" s="111"/>
+      <c r="I14" s="111"/>
+      <c r="J14" s="111"/>
     </row>
     <row r="15" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="107"/>
-      <c r="B15" s="109" t="s">
+      <c r="A15" s="105"/>
+      <c r="B15" s="107" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="104"/>
-      <c r="D15" s="104"/>
-      <c r="E15" s="104"/>
-      <c r="F15" s="105"/>
-      <c r="G15" s="105"/>
-      <c r="H15" s="105"/>
-      <c r="I15" s="105"/>
-      <c r="J15" s="105"/>
+      <c r="C15" s="108"/>
+      <c r="D15" s="108"/>
+      <c r="E15" s="108"/>
+      <c r="F15" s="111"/>
+      <c r="G15" s="111"/>
+      <c r="H15" s="111"/>
+      <c r="I15" s="111"/>
+      <c r="J15" s="111"/>
     </row>
     <row r="16" spans="1:10" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="107"/>
-      <c r="B16" s="109" t="s">
+      <c r="A16" s="105"/>
+      <c r="B16" s="107" t="s">
         <v>22</v>
       </c>
-      <c r="C16" s="104"/>
-      <c r="D16" s="104"/>
-      <c r="E16" s="104"/>
-      <c r="F16" s="105"/>
-      <c r="G16" s="105"/>
-      <c r="H16" s="105"/>
-      <c r="I16" s="105"/>
-      <c r="J16" s="105"/>
+      <c r="C16" s="108"/>
+      <c r="D16" s="108"/>
+      <c r="E16" s="108"/>
+      <c r="F16" s="111"/>
+      <c r="G16" s="111"/>
+      <c r="H16" s="111"/>
+      <c r="I16" s="111"/>
+      <c r="J16" s="111"/>
     </row>
     <row r="17" spans="1:10" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="107"/>
-      <c r="B17" s="110" t="s">
+      <c r="A17" s="105"/>
+      <c r="B17" s="109" t="s">
         <v>23</v>
       </c>
-      <c r="C17" s="111"/>
-      <c r="D17" s="111"/>
-      <c r="E17" s="111"/>
-      <c r="F17" s="105"/>
-      <c r="G17" s="105"/>
-      <c r="H17" s="105"/>
-      <c r="I17" s="105"/>
-      <c r="J17" s="105"/>
+      <c r="C17" s="110"/>
+      <c r="D17" s="110"/>
+      <c r="E17" s="110"/>
+      <c r="F17" s="111"/>
+      <c r="G17" s="111"/>
+      <c r="H17" s="111"/>
+      <c r="I17" s="111"/>
+      <c r="J17" s="111"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="2"/>
-      <c r="B18" s="106"/>
-      <c r="C18" s="106"/>
-      <c r="D18" s="106"/>
+      <c r="B18" s="104"/>
+      <c r="C18" s="104"/>
+      <c r="D18" s="104"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
@@ -2011,9 +2011,9 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="2"/>
-      <c r="B19" s="104"/>
-      <c r="C19" s="104"/>
-      <c r="D19" s="104"/>
+      <c r="B19" s="108"/>
+      <c r="C19" s="108"/>
+      <c r="D19" s="108"/>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
@@ -2023,9 +2023,9 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="2"/>
-      <c r="B20" s="104"/>
-      <c r="C20" s="104"/>
-      <c r="D20" s="104"/>
+      <c r="B20" s="108"/>
+      <c r="C20" s="108"/>
+      <c r="D20" s="108"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
@@ -2035,9 +2035,9 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="2"/>
-      <c r="B21" s="104"/>
-      <c r="C21" s="104"/>
-      <c r="D21" s="104"/>
+      <c r="B21" s="108"/>
+      <c r="C21" s="108"/>
+      <c r="D21" s="108"/>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
@@ -2047,9 +2047,9 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" s="2"/>
-      <c r="B22" s="104"/>
-      <c r="C22" s="104"/>
-      <c r="D22" s="104"/>
+      <c r="B22" s="108"/>
+      <c r="C22" s="108"/>
+      <c r="D22" s="108"/>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
@@ -2059,9 +2059,9 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="2"/>
-      <c r="B23" s="104"/>
-      <c r="C23" s="104"/>
-      <c r="D23" s="104"/>
+      <c r="B23" s="108"/>
+      <c r="C23" s="108"/>
+      <c r="D23" s="108"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
@@ -2071,9 +2071,9 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="2"/>
-      <c r="B24" s="104"/>
-      <c r="C24" s="104"/>
-      <c r="D24" s="104"/>
+      <c r="B24" s="108"/>
+      <c r="C24" s="108"/>
+      <c r="D24" s="108"/>
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
@@ -2083,9 +2083,9 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="2"/>
-      <c r="B25" s="104"/>
-      <c r="C25" s="104"/>
-      <c r="D25" s="104"/>
+      <c r="B25" s="108"/>
+      <c r="C25" s="108"/>
+      <c r="D25" s="108"/>
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
@@ -2095,9 +2095,9 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="2"/>
-      <c r="B26" s="104"/>
-      <c r="C26" s="104"/>
-      <c r="D26" s="104"/>
+      <c r="B26" s="108"/>
+      <c r="C26" s="108"/>
+      <c r="D26" s="108"/>
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
@@ -2119,18 +2119,6 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="A13:A17"/>
-    <mergeCell ref="B13:E13"/>
-    <mergeCell ref="B14:E14"/>
-    <mergeCell ref="B15:E15"/>
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="B17:E17"/>
-    <mergeCell ref="F13:F17"/>
-    <mergeCell ref="G13:G17"/>
-    <mergeCell ref="H13:H17"/>
-    <mergeCell ref="I13:I17"/>
-    <mergeCell ref="J13:J17"/>
     <mergeCell ref="B25:D25"/>
     <mergeCell ref="B26:D26"/>
     <mergeCell ref="B19:D19"/>
@@ -2139,6 +2127,18 @@
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="B24:D24"/>
+    <mergeCell ref="F13:F17"/>
+    <mergeCell ref="G13:G17"/>
+    <mergeCell ref="H13:H17"/>
+    <mergeCell ref="I13:I17"/>
+    <mergeCell ref="J13:J17"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="A13:A17"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="B17:E17"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="H7" r:id="rId1" display="https://github.com/CloudLabsAI-Azure/AI-Agents-using-Microsoft-Frameworks" xr:uid="{DC729D3C-6769-4CCA-B76B-0365C00D9A0F}"/>
@@ -2163,17 +2163,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="26" x14ac:dyDescent="0.6">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="75" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="98"/>
-      <c r="C1" s="98"/>
-      <c r="D1" s="98"/>
-      <c r="E1" s="98"/>
-      <c r="F1" s="98"/>
-      <c r="G1" s="98"/>
-      <c r="H1" s="98"/>
-      <c r="I1" s="98"/>
+      <c r="B1" s="76"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="76"/>
+      <c r="E1" s="76"/>
+      <c r="F1" s="76"/>
+      <c r="G1" s="76"/>
+      <c r="H1" s="76"/>
+      <c r="I1" s="76"/>
       <c r="J1" s="1"/>
       <c r="K1" s="2"/>
       <c r="L1" s="2"/>
@@ -2184,19 +2184,19 @@
       <c r="Q1" s="2"/>
     </row>
     <row r="2" spans="1:17" ht="16" x14ac:dyDescent="0.4">
-      <c r="A2" s="99" t="s">
+      <c r="A2" s="77" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="100"/>
-      <c r="C2" s="101"/>
+      <c r="B2" s="78"/>
+      <c r="C2" s="79"/>
       <c r="D2" s="3">
         <v>6</v>
       </c>
-      <c r="E2" s="102"/>
-      <c r="F2" s="103"/>
-      <c r="G2" s="103"/>
-      <c r="H2" s="103"/>
-      <c r="I2" s="103"/>
+      <c r="E2" s="80"/>
+      <c r="F2" s="81"/>
+      <c r="G2" s="81"/>
+      <c r="H2" s="81"/>
+      <c r="I2" s="81"/>
       <c r="J2" s="1"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
@@ -2207,19 +2207,19 @@
       <c r="Q2" s="2"/>
     </row>
     <row r="3" spans="1:17" ht="16" x14ac:dyDescent="0.4">
-      <c r="A3" s="92" t="s">
+      <c r="A3" s="70" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="93"/>
-      <c r="C3" s="94"/>
+      <c r="B3" s="71"/>
+      <c r="C3" s="72"/>
       <c r="D3" s="4">
         <v>6</v>
       </c>
-      <c r="E3" s="95"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="96"/>
-      <c r="H3" s="96"/>
-      <c r="I3" s="96"/>
+      <c r="E3" s="73"/>
+      <c r="F3" s="74"/>
+      <c r="G3" s="74"/>
+      <c r="H3" s="74"/>
+      <c r="I3" s="74"/>
       <c r="J3" s="1"/>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
@@ -2230,20 +2230,20 @@
       <c r="Q3" s="2"/>
     </row>
     <row r="4" spans="1:17" ht="16" x14ac:dyDescent="0.4">
-      <c r="A4" s="92" t="s">
+      <c r="A4" s="70" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="93"/>
-      <c r="C4" s="94"/>
+      <c r="B4" s="71"/>
+      <c r="C4" s="72"/>
       <c r="D4" s="4">
         <f>'Overall-cost'!F7</f>
         <v>1</v>
       </c>
-      <c r="E4" s="95"/>
-      <c r="F4" s="96"/>
-      <c r="G4" s="96"/>
-      <c r="H4" s="96"/>
-      <c r="I4" s="96"/>
+      <c r="E4" s="73"/>
+      <c r="F4" s="74"/>
+      <c r="G4" s="74"/>
+      <c r="H4" s="74"/>
+      <c r="I4" s="74"/>
       <c r="J4" s="1"/>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
@@ -2254,15 +2254,15 @@
       <c r="Q4" s="2"/>
     </row>
     <row r="5" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="79"/>
-      <c r="B5" s="80"/>
-      <c r="C5" s="80"/>
-      <c r="D5" s="80"/>
-      <c r="E5" s="80"/>
-      <c r="F5" s="80"/>
-      <c r="G5" s="80"/>
-      <c r="H5" s="80"/>
-      <c r="I5" s="80"/>
+      <c r="A5" s="91"/>
+      <c r="B5" s="92"/>
+      <c r="C5" s="92"/>
+      <c r="D5" s="92"/>
+      <c r="E5" s="92"/>
+      <c r="F5" s="92"/>
+      <c r="G5" s="92"/>
+      <c r="H5" s="92"/>
+      <c r="I5" s="92"/>
       <c r="J5" s="1"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
@@ -2273,17 +2273,17 @@
       <c r="Q5" s="2"/>
     </row>
     <row r="6" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="81" t="s">
+      <c r="A6" s="93" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="82"/>
-      <c r="C6" s="82"/>
-      <c r="D6" s="82"/>
-      <c r="E6" s="82"/>
-      <c r="F6" s="82"/>
-      <c r="G6" s="82"/>
-      <c r="H6" s="82"/>
-      <c r="I6" s="82"/>
+      <c r="B6" s="94"/>
+      <c r="C6" s="94"/>
+      <c r="D6" s="94"/>
+      <c r="E6" s="94"/>
+      <c r="F6" s="94"/>
+      <c r="G6" s="94"/>
+      <c r="H6" s="94"/>
+      <c r="I6" s="94"/>
       <c r="J6" s="1"/>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
@@ -2331,7 +2331,7 @@
       <c r="Q7" s="2"/>
     </row>
     <row r="8" spans="1:17" ht="87.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="89" t="s">
+      <c r="A8" s="101" t="s">
         <v>51</v>
       </c>
       <c r="B8" s="10" t="s">
@@ -2343,7 +2343,9 @@
       <c r="D8" s="11">
         <v>1</v>
       </c>
-      <c r="E8" s="44"/>
+      <c r="E8" s="44">
+        <v>137.24</v>
+      </c>
       <c r="F8" s="13">
         <v>0</v>
       </c>
@@ -2352,7 +2354,7 @@
       </c>
       <c r="H8" s="43">
         <f>IF(D8=0,(E8/720)*D$2*G8+F8*G8,(E8/720)*D$3*G8+F8*G8)</f>
-        <v>0</v>
+        <v>1.1436666666666668</v>
       </c>
       <c r="I8" s="14"/>
       <c r="J8" s="1"/>
@@ -2365,17 +2367,19 @@
       <c r="Q8" s="2"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A9" s="90"/>
+      <c r="A9" s="102"/>
       <c r="B9" s="15" t="s">
         <v>38</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D9" s="11">
         <v>0</v>
       </c>
-      <c r="E9" s="44"/>
+      <c r="E9" s="44">
+        <v>19.71</v>
+      </c>
       <c r="F9" s="13">
         <v>0</v>
       </c>
@@ -2384,7 +2388,7 @@
       </c>
       <c r="H9" s="43">
         <f t="shared" ref="H9:H14" si="0">IF(D9=0,(E9/720)*D$2*G9+F9*G9,(E9/720)*D$3*G9+F9*G9)</f>
-        <v>0</v>
+        <v>0.16425000000000001</v>
       </c>
       <c r="I9" s="14"/>
       <c r="J9" s="1"/>
@@ -2397,7 +2401,7 @@
       <c r="Q9" s="2"/>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A10" s="90"/>
+      <c r="A10" s="102"/>
       <c r="B10" s="15" t="s">
         <v>39</v>
       </c>
@@ -2431,7 +2435,7 @@
       <c r="Q10" s="1"/>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A11" s="90"/>
+      <c r="A11" s="102"/>
       <c r="B11" s="15" t="s">
         <v>41</v>
       </c>
@@ -2463,7 +2467,7 @@
       <c r="Q11" s="2"/>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A12" s="90"/>
+      <c r="A12" s="102"/>
       <c r="B12" s="15" t="s">
         <v>42</v>
       </c>
@@ -2495,7 +2499,7 @@
       <c r="Q12" s="1"/>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A13" s="90"/>
+      <c r="A13" s="102"/>
       <c r="B13" s="15" t="s">
         <v>43</v>
       </c>
@@ -2527,12 +2531,12 @@
       <c r="Q13" s="1"/>
     </row>
     <row r="14" spans="1:17" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="90"/>
+      <c r="A14" s="102"/>
       <c r="B14" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>57</v>
       </c>
       <c r="D14" s="11">
         <v>0</v>
@@ -2561,7 +2565,7 @@
       <c r="Q14" s="1"/>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A15" s="90"/>
+      <c r="A15" s="102"/>
       <c r="B15" s="18"/>
       <c r="C15" s="19"/>
       <c r="D15" s="11"/>
@@ -2580,7 +2584,7 @@
       <c r="Q15" s="1"/>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A16" s="90"/>
+      <c r="A16" s="102"/>
       <c r="B16" s="13"/>
       <c r="C16" s="13"/>
       <c r="D16" s="13"/>
@@ -2599,7 +2603,7 @@
       <c r="Q16" s="1"/>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A17" s="91"/>
+      <c r="A17" s="103"/>
       <c r="B17" s="65" t="s">
         <v>44</v>
       </c>
@@ -2610,7 +2614,7 @@
       <c r="G17" s="67"/>
       <c r="H17" s="68">
         <f>SUM(H8:H14)</f>
-        <v>0.50541666666666663</v>
+        <v>1.8133333333333335</v>
       </c>
       <c r="I17" s="69"/>
       <c r="J17" s="1"/>
@@ -2623,18 +2627,18 @@
       <c r="Q17" s="1"/>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A18" s="83" t="s">
+      <c r="A18" s="95" t="s">
         <v>45</v>
       </c>
-      <c r="B18" s="84"/>
-      <c r="C18" s="84"/>
-      <c r="D18" s="84"/>
-      <c r="E18" s="84"/>
-      <c r="F18" s="84"/>
-      <c r="G18" s="85"/>
+      <c r="B18" s="96"/>
+      <c r="C18" s="96"/>
+      <c r="D18" s="96"/>
+      <c r="E18" s="96"/>
+      <c r="F18" s="96"/>
+      <c r="G18" s="97"/>
       <c r="H18" s="47">
         <f>H17*D4</f>
-        <v>0.50541666666666663</v>
+        <v>1.8133333333333335</v>
       </c>
       <c r="I18" s="20"/>
       <c r="J18" s="2"/>
@@ -2685,11 +2689,11 @@
       <c r="Q20" s="2"/>
     </row>
     <row r="21" spans="1:17" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="86" t="s">
+      <c r="A21" s="98" t="s">
         <v>46</v>
       </c>
-      <c r="B21" s="87"/>
-      <c r="C21" s="88"/>
+      <c r="B21" s="99"/>
+      <c r="C21" s="100"/>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
@@ -2706,11 +2710,11 @@
       <c r="Q21" s="2"/>
     </row>
     <row r="22" spans="1:17" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="70" t="s">
+      <c r="A22" s="82" t="s">
         <v>47</v>
       </c>
-      <c r="B22" s="71"/>
-      <c r="C22" s="72"/>
+      <c r="B22" s="83"/>
+      <c r="C22" s="84"/>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
@@ -2727,11 +2731,11 @@
       <c r="Q22" s="2"/>
     </row>
     <row r="23" spans="1:17" ht="58" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="70" t="s">
+      <c r="A23" s="82" t="s">
         <v>48</v>
       </c>
-      <c r="B23" s="71"/>
-      <c r="C23" s="72"/>
+      <c r="B23" s="83"/>
+      <c r="C23" s="84"/>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
@@ -2748,11 +2752,11 @@
       <c r="Q23" s="2"/>
     </row>
     <row r="24" spans="1:17" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="70" t="s">
+      <c r="A24" s="82" t="s">
         <v>49</v>
       </c>
-      <c r="B24" s="71"/>
-      <c r="C24" s="72"/>
+      <c r="B24" s="83"/>
+      <c r="C24" s="84"/>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
@@ -2769,11 +2773,11 @@
       <c r="Q24" s="2"/>
     </row>
     <row r="25" spans="1:17" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="73" t="s">
+      <c r="A25" s="85" t="s">
         <v>50</v>
       </c>
-      <c r="B25" s="74"/>
-      <c r="C25" s="75"/>
+      <c r="B25" s="86"/>
+      <c r="C25" s="87"/>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
@@ -2790,9 +2794,9 @@
       <c r="Q25" s="2"/>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A26" s="76"/>
-      <c r="B26" s="77"/>
-      <c r="C26" s="78"/>
+      <c r="A26" s="88"/>
+      <c r="B26" s="89"/>
+      <c r="C26" s="90"/>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
@@ -2815,13 +2819,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="E4:I4"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="E2:I2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="E3:I3"/>
     <mergeCell ref="A24:C24"/>
     <mergeCell ref="A25:C25"/>
     <mergeCell ref="A26:C26"/>
@@ -2832,18 +2829,30 @@
     <mergeCell ref="A22:C22"/>
     <mergeCell ref="A23:C23"/>
     <mergeCell ref="A8:A17"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="E4:I4"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="E2:I2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="E3:I3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1a6be2e8-895c-4bca-ac32-df7929f4fc94">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="32c83a25-b22d-480d-8556-52adf92b9d23" xsi:nil="true"/>
+    <ExportedDate xmlns="1a6be2e8-895c-4bca-ac32-df7929f4fc94" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3125,23 +3134,22 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1a6be2e8-895c-4bca-ac32-df7929f4fc94">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="32c83a25-b22d-480d-8556-52adf92b9d23" xsi:nil="true"/>
-    <ExportedDate xmlns="1a6be2e8-895c-4bca-ac32-df7929f4fc94" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3DDCD5B0-9850-4CCE-A29D-FDDC2EBA3C08}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FACEAE82-5710-4A25-B94D-AFE68277E1C5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="1a6be2e8-895c-4bca-ac32-df7929f4fc94"/>
+    <ds:schemaRef ds:uri="32c83a25-b22d-480d-8556-52adf92b9d23"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3167,13 +3175,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FACEAE82-5710-4A25-B94D-AFE68277E1C5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3DDCD5B0-9850-4CCE-A29D-FDDC2EBA3C08}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="1a6be2e8-895c-4bca-ac32-df7929f4fc94"/>
-    <ds:schemaRef ds:uri="32c83a25-b22d-480d-8556-52adf92b9d23"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>